<commit_message>
Standardize demo seed data
</commit_message>
<xml_diff>
--- a/ornek-veriler/ogretmen-aktarim-sablonu.xlsx
+++ b/ornek-veriler/ogretmen-aktarim-sablonu.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44">
-  <si>
-    <t>ogretmen-aktarim-sablonu</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+  <si>
+    <t>ogretmen-aktarim-sablonu (1)</t>
   </si>
   <si>
     <t>ad</t>
@@ -22,19 +22,13 @@
     <t>soyad</t>
   </si>
   <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>telefon</t>
-  </si>
-  <si>
     <t>brans</t>
   </si>
   <si>
     <t>atanacak_sinif</t>
   </si>
   <si>
-    <t>not</t>
+    <t>ders</t>
   </si>
   <si>
     <t>Ayse</t>
@@ -43,74 +37,27 @@
     <t>Hoca</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>ayse@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Matematik</t>
   </si>
   <si>
     <t>8 LGS A</t>
   </si>
   <si>
-    <t>Branş öğretmeni</t>
-  </si>
-  <si>
     <t>Fatma</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>fatma@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Türkçe</t>
   </si>
   <si>
     <t>Mehmet</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>mehmet@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Sosyal Bilgiler</t>
   </si>
   <si>
     <t>Hikmet</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>hikmet@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Fen Bilimleri</t>
   </si>
   <si>
@@ -120,117 +67,37 @@
     <t>Ali</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>ali@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Din Kültürü</t>
   </si>
   <si>
     <t>Ahmet</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>ahmet@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>İngilizce</t>
   </si>
   <si>
     <t>Ömer</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>ömer@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>8 LGS C</t>
   </si>
   <si>
     <t>Nuri</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>nuri@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Hasan</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>hasan@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Cem</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>cem@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>8 LGS D</t>
   </si>
   <si>
     <t>Sultan</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>sultan@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Barış</t>
-  </si>
-  <si>
-    <t>baris@example.test</t>
   </si>
 </sst>
 </file>
@@ -240,7 +107,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -253,12 +120,6 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <u val="single"/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
@@ -403,7 +264,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -425,9 +286,6 @@
     <xf numFmtId="49" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
@@ -437,7 +295,13 @@
     <xf numFmtId="49" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1492,17 +1356,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:G14"/>
+  <dimension ref="A2:E18"/>
   <sheetFormatPr defaultColWidth="8.33333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="5.35156" style="1" customWidth="1"/>
     <col min="2" max="2" width="6.35156" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5391" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6719" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.0781" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13" style="1" customWidth="1"/>
-    <col min="7" max="7" width="13.8516" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.35156" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.35156" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.35156" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.35156" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
@@ -1513,8 +1375,6 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" t="s" s="3">
@@ -1532,306 +1392,253 @@
       <c r="E2" t="s" s="3">
         <v>5</v>
       </c>
-      <c r="F2" t="s" s="3">
-        <v>6</v>
-      </c>
-      <c r="G2" t="s" s="3">
-        <v>7</v>
-      </c>
     </row>
     <row r="3" ht="20.25" customHeight="1">
       <c r="A3" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s" s="5">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="6">
         <v>8</v>
       </c>
-      <c r="B3" t="s" s="5">
+      <c r="D3" t="s" s="6">
         <v>9</v>
       </c>
-      <c r="C3" t="s" s="6">
+      <c r="E3" t="s" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" ht="20.05" customHeight="1">
+      <c r="A4" t="s" s="7">
         <v>10</v>
       </c>
-      <c r="D3" s="7">
-        <v>5551112233</v>
-      </c>
-      <c r="E3" t="s" s="6">
+      <c r="B4" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s" s="9">
         <v>11</v>
       </c>
-      <c r="F3" t="s" s="6">
+      <c r="D4" t="s" s="9">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" ht="20.05" customHeight="1">
+      <c r="A5" t="s" s="7">
         <v>12</v>
       </c>
-      <c r="G3" t="s" s="6">
+      <c r="B5" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" t="s" s="8">
+      <c r="D5" t="s" s="9">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s" s="9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" ht="20.05" customHeight="1">
+      <c r="A6" t="s" s="7">
         <v>14</v>
       </c>
-      <c r="B4" t="s" s="9">
+      <c r="B6" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s" s="9">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s" s="9">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" ht="20.05" customHeight="1">
+      <c r="A7" t="s" s="7">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s" s="9">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s" s="9">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s" s="9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" ht="20.05" customHeight="1">
+      <c r="A8" t="s" s="7">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s" s="9">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s" s="9">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="20.05" customHeight="1">
+      <c r="A9" t="s" s="7">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s" s="9">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s" s="9">
+        <v>22</v>
+      </c>
+      <c r="E9" t="s" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" ht="20.05" customHeight="1">
+      <c r="A10" t="s" s="7">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s" s="9">
+        <v>22</v>
+      </c>
+      <c r="E10" t="s" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" ht="20.05" customHeight="1">
+      <c r="A11" t="s" s="7">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s" s="9">
+        <v>13</v>
+      </c>
+      <c r="D11" t="s" s="9">
+        <v>22</v>
+      </c>
+      <c r="E11" t="s" s="9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" ht="20.05" customHeight="1">
+      <c r="A12" t="s" s="7">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s" s="9">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s" s="9">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" ht="20.05" customHeight="1">
+      <c r="A13" t="s" s="7">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s" s="9">
+        <v>18</v>
+      </c>
+      <c r="D13" t="s" s="9">
+        <v>26</v>
+      </c>
+      <c r="E13" t="s" s="9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" ht="20.05" customHeight="1">
+      <c r="A14" t="s" s="7">
+        <v>28</v>
+      </c>
+      <c r="B14" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s" s="9">
+        <v>20</v>
+      </c>
+      <c r="D14" t="s" s="9">
+        <v>26</v>
+      </c>
+      <c r="E14" t="s" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" ht="20.05" customHeight="1">
+      <c r="A15" t="s" s="7">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s" s="9">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s" s="9">
         <v>9</v>
       </c>
-      <c r="C4" t="s" s="10">
-        <v>15</v>
-      </c>
-      <c r="D4" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E4" t="s" s="10">
-        <v>16</v>
-      </c>
-      <c r="F4" t="s" s="10">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" t="s" s="8">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s" s="10">
-        <v>18</v>
-      </c>
-      <c r="D5" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E5" t="s" s="10">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s" s="10">
-        <v>12</v>
-      </c>
-      <c r="G5" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" t="s" s="8">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s" s="10">
-        <v>21</v>
-      </c>
-      <c r="D6" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E6" t="s" s="10">
-        <v>22</v>
-      </c>
-      <c r="F6" t="s" s="10">
-        <v>23</v>
-      </c>
-      <c r="G6" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" t="s" s="8">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s" s="10">
-        <v>25</v>
-      </c>
-      <c r="D7" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E7" t="s" s="10">
-        <v>26</v>
-      </c>
-      <c r="F7" t="s" s="10">
-        <v>23</v>
-      </c>
-      <c r="G7" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" t="s" s="8">
-        <v>27</v>
-      </c>
-      <c r="B8" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s" s="10">
-        <v>28</v>
-      </c>
-      <c r="D8" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E8" t="s" s="10">
-        <v>29</v>
-      </c>
-      <c r="F8" t="s" s="10">
-        <v>23</v>
-      </c>
-      <c r="G8" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" t="s" s="8">
-        <v>30</v>
-      </c>
-      <c r="B9" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s" s="10">
-        <v>31</v>
-      </c>
-      <c r="D9" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E9" t="s" s="10">
-        <v>11</v>
-      </c>
-      <c r="F9" t="s" s="10">
-        <v>32</v>
-      </c>
-      <c r="G9" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" t="s" s="8">
-        <v>33</v>
-      </c>
-      <c r="B10" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s" s="10">
-        <v>34</v>
-      </c>
-      <c r="D10" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E10" t="s" s="10">
-        <v>16</v>
-      </c>
-      <c r="F10" t="s" s="10">
-        <v>32</v>
-      </c>
-      <c r="G10" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" t="s" s="8">
-        <v>35</v>
-      </c>
-      <c r="B11" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s" s="10">
-        <v>36</v>
-      </c>
-      <c r="D11" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E11" t="s" s="10">
-        <v>19</v>
-      </c>
-      <c r="F11" t="s" s="10">
-        <v>32</v>
-      </c>
-      <c r="G11" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" t="s" s="8">
-        <v>37</v>
-      </c>
-      <c r="B12" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C12" t="s" s="10">
-        <v>38</v>
-      </c>
-      <c r="D12" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E12" t="s" s="10">
-        <v>22</v>
-      </c>
-      <c r="F12" t="s" s="10">
-        <v>39</v>
-      </c>
-      <c r="G12" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" t="s" s="8">
-        <v>40</v>
-      </c>
-      <c r="B13" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s" s="10">
-        <v>41</v>
-      </c>
-      <c r="D13" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E13" t="s" s="10">
-        <v>26</v>
-      </c>
-      <c r="F13" t="s" s="10">
-        <v>39</v>
-      </c>
-      <c r="G13" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" t="s" s="8">
-        <v>42</v>
-      </c>
-      <c r="B14" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C14" t="s" s="10">
-        <v>43</v>
-      </c>
-      <c r="D14" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E14" t="s" s="10">
-        <v>29</v>
-      </c>
-      <c r="F14" t="s" s="10">
-        <v>39</v>
-      </c>
-      <c r="G14" t="s" s="10">
-        <v>13</v>
-      </c>
+      <c r="E15" t="s" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" ht="20.05" customHeight="1">
+      <c r="A16" s="10"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+    </row>
+    <row r="17" ht="20.05" customHeight="1">
+      <c r="A17" s="10"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+    </row>
+    <row r="18" ht="20.05" customHeight="1">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" location="" tooltip="" display="ayse@example.test"/>
-    <hyperlink ref="C4" r:id="rId2" location="" tooltip="" display="fatma@example.test"/>
-    <hyperlink ref="C5" r:id="rId3" location="" tooltip="" display="mehmet@example.test"/>
-    <hyperlink ref="C6" r:id="rId4" location="" tooltip="" display="hikmet@example.test"/>
-    <hyperlink ref="C7" r:id="rId5" location="" tooltip="" display="ali@example.test"/>
-    <hyperlink ref="C8" r:id="rId6" location="" tooltip="" display="ahmet@example.test"/>
-    <hyperlink ref="C9" r:id="rId7" location="" tooltip="" display="ömer@example.test"/>
-    <hyperlink ref="C10" r:id="rId8" location="" tooltip="" display="nuri@example.test"/>
-    <hyperlink ref="C11" r:id="rId9" location="" tooltip="" display="hasan@example.test"/>
-    <hyperlink ref="C12" r:id="rId10" location="" tooltip="" display="cem@example.test"/>
-    <hyperlink ref="C13" r:id="rId11" location="" tooltip="" display="sultan@example.test"/>
-  </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>

</xml_diff>

<commit_message>
[codex] Standardize demo seed data (#12)
* Standardize demo seed data

* Align UX baseline with exam answer key flow

* Clean Next artifacts before web type checks

* Align RBAC exam test with answer key creation

* Prevent duplicate first admin tenant membership
</commit_message>
<xml_diff>
--- a/ornek-veriler/ogretmen-aktarim-sablonu.xlsx
+++ b/ornek-veriler/ogretmen-aktarim-sablonu.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="44">
-  <si>
-    <t>ogretmen-aktarim-sablonu</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+  <si>
+    <t>ogretmen-aktarim-sablonu (1)</t>
   </si>
   <si>
     <t>ad</t>
@@ -22,19 +22,13 @@
     <t>soyad</t>
   </si>
   <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>telefon</t>
-  </si>
-  <si>
     <t>brans</t>
   </si>
   <si>
     <t>atanacak_sinif</t>
   </si>
   <si>
-    <t>not</t>
+    <t>ders</t>
   </si>
   <si>
     <t>Ayse</t>
@@ -43,74 +37,27 @@
     <t>Hoca</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>ayse@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Matematik</t>
   </si>
   <si>
     <t>8 LGS A</t>
   </si>
   <si>
-    <t>Branş öğretmeni</t>
-  </si>
-  <si>
     <t>Fatma</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>fatma@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Türkçe</t>
   </si>
   <si>
     <t>Mehmet</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>mehmet@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Sosyal Bilgiler</t>
   </si>
   <si>
     <t>Hikmet</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>hikmet@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Fen Bilimleri</t>
   </si>
   <si>
@@ -120,117 +67,37 @@
     <t>Ali</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>ali@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Din Kültürü</t>
   </si>
   <si>
     <t>Ahmet</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>ahmet@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>İngilizce</t>
   </si>
   <si>
     <t>Ömer</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>ömer@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>8 LGS C</t>
   </si>
   <si>
     <t>Nuri</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>nuri@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Hasan</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>hasan@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Cem</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>cem@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>8 LGS D</t>
   </si>
   <si>
     <t>Sultan</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>sultan@example.test</t>
-    </r>
-  </si>
-  <si>
     <t>Barış</t>
-  </si>
-  <si>
-    <t>baris@example.test</t>
   </si>
 </sst>
 </file>
@@ -240,7 +107,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -253,12 +120,6 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <u val="single"/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
@@ -403,7 +264,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -425,9 +286,6 @@
     <xf numFmtId="49" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
@@ -437,7 +295,13 @@
     <xf numFmtId="49" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1492,17 +1356,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:G14"/>
+  <dimension ref="A2:E18"/>
   <sheetFormatPr defaultColWidth="8.33333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="5.35156" style="1" customWidth="1"/>
     <col min="2" max="2" width="6.35156" style="1" customWidth="1"/>
-    <col min="3" max="3" width="23.5391" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6719" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.0781" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13" style="1" customWidth="1"/>
-    <col min="7" max="7" width="13.8516" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.35156" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.35156" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.35156" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.35156" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.65" customHeight="1">
@@ -1513,8 +1375,6 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
     </row>
     <row r="2" ht="20.25" customHeight="1">
       <c r="A2" t="s" s="3">
@@ -1532,306 +1392,253 @@
       <c r="E2" t="s" s="3">
         <v>5</v>
       </c>
-      <c r="F2" t="s" s="3">
-        <v>6</v>
-      </c>
-      <c r="G2" t="s" s="3">
-        <v>7</v>
-      </c>
     </row>
     <row r="3" ht="20.25" customHeight="1">
       <c r="A3" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s" s="5">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="6">
         <v>8</v>
       </c>
-      <c r="B3" t="s" s="5">
+      <c r="D3" t="s" s="6">
         <v>9</v>
       </c>
-      <c r="C3" t="s" s="6">
+      <c r="E3" t="s" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" ht="20.05" customHeight="1">
+      <c r="A4" t="s" s="7">
         <v>10</v>
       </c>
-      <c r="D3" s="7">
-        <v>5551112233</v>
-      </c>
-      <c r="E3" t="s" s="6">
+      <c r="B4" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s" s="9">
         <v>11</v>
       </c>
-      <c r="F3" t="s" s="6">
+      <c r="D4" t="s" s="9">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" ht="20.05" customHeight="1">
+      <c r="A5" t="s" s="7">
         <v>12</v>
       </c>
-      <c r="G3" t="s" s="6">
+      <c r="B5" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" t="s" s="8">
+      <c r="D5" t="s" s="9">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s" s="9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" ht="20.05" customHeight="1">
+      <c r="A6" t="s" s="7">
         <v>14</v>
       </c>
-      <c r="B4" t="s" s="9">
+      <c r="B6" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s" s="9">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s" s="9">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" ht="20.05" customHeight="1">
+      <c r="A7" t="s" s="7">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s" s="9">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s" s="9">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s" s="9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" ht="20.05" customHeight="1">
+      <c r="A8" t="s" s="7">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s" s="9">
+        <v>20</v>
+      </c>
+      <c r="D8" t="s" s="9">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="20.05" customHeight="1">
+      <c r="A9" t="s" s="7">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s" s="9">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s" s="9">
+        <v>22</v>
+      </c>
+      <c r="E9" t="s" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" ht="20.05" customHeight="1">
+      <c r="A10" t="s" s="7">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s" s="9">
+        <v>22</v>
+      </c>
+      <c r="E10" t="s" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" ht="20.05" customHeight="1">
+      <c r="A11" t="s" s="7">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s" s="9">
+        <v>13</v>
+      </c>
+      <c r="D11" t="s" s="9">
+        <v>22</v>
+      </c>
+      <c r="E11" t="s" s="9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" ht="20.05" customHeight="1">
+      <c r="A12" t="s" s="7">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s" s="9">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s" s="9">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" ht="20.05" customHeight="1">
+      <c r="A13" t="s" s="7">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s" s="9">
+        <v>18</v>
+      </c>
+      <c r="D13" t="s" s="9">
+        <v>26</v>
+      </c>
+      <c r="E13" t="s" s="9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" ht="20.05" customHeight="1">
+      <c r="A14" t="s" s="7">
+        <v>28</v>
+      </c>
+      <c r="B14" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s" s="9">
+        <v>20</v>
+      </c>
+      <c r="D14" t="s" s="9">
+        <v>26</v>
+      </c>
+      <c r="E14" t="s" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" ht="20.05" customHeight="1">
+      <c r="A15" t="s" s="7">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s" s="8">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s" s="9">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s" s="9">
         <v>9</v>
       </c>
-      <c r="C4" t="s" s="10">
-        <v>15</v>
-      </c>
-      <c r="D4" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E4" t="s" s="10">
-        <v>16</v>
-      </c>
-      <c r="F4" t="s" s="10">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" t="s" s="8">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s" s="10">
-        <v>18</v>
-      </c>
-      <c r="D5" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E5" t="s" s="10">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s" s="10">
-        <v>12</v>
-      </c>
-      <c r="G5" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" t="s" s="8">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s" s="10">
-        <v>21</v>
-      </c>
-      <c r="D6" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E6" t="s" s="10">
-        <v>22</v>
-      </c>
-      <c r="F6" t="s" s="10">
-        <v>23</v>
-      </c>
-      <c r="G6" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" t="s" s="8">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s" s="10">
-        <v>25</v>
-      </c>
-      <c r="D7" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E7" t="s" s="10">
-        <v>26</v>
-      </c>
-      <c r="F7" t="s" s="10">
-        <v>23</v>
-      </c>
-      <c r="G7" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" t="s" s="8">
-        <v>27</v>
-      </c>
-      <c r="B8" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s" s="10">
-        <v>28</v>
-      </c>
-      <c r="D8" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E8" t="s" s="10">
-        <v>29</v>
-      </c>
-      <c r="F8" t="s" s="10">
-        <v>23</v>
-      </c>
-      <c r="G8" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" t="s" s="8">
-        <v>30</v>
-      </c>
-      <c r="B9" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s" s="10">
-        <v>31</v>
-      </c>
-      <c r="D9" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E9" t="s" s="10">
-        <v>11</v>
-      </c>
-      <c r="F9" t="s" s="10">
-        <v>32</v>
-      </c>
-      <c r="G9" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" t="s" s="8">
-        <v>33</v>
-      </c>
-      <c r="B10" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s" s="10">
-        <v>34</v>
-      </c>
-      <c r="D10" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E10" t="s" s="10">
-        <v>16</v>
-      </c>
-      <c r="F10" t="s" s="10">
-        <v>32</v>
-      </c>
-      <c r="G10" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" ht="20.05" customHeight="1">
-      <c r="A11" t="s" s="8">
-        <v>35</v>
-      </c>
-      <c r="B11" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s" s="10">
-        <v>36</v>
-      </c>
-      <c r="D11" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E11" t="s" s="10">
-        <v>19</v>
-      </c>
-      <c r="F11" t="s" s="10">
-        <v>32</v>
-      </c>
-      <c r="G11" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" t="s" s="8">
-        <v>37</v>
-      </c>
-      <c r="B12" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C12" t="s" s="10">
-        <v>38</v>
-      </c>
-      <c r="D12" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E12" t="s" s="10">
-        <v>22</v>
-      </c>
-      <c r="F12" t="s" s="10">
-        <v>39</v>
-      </c>
-      <c r="G12" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" t="s" s="8">
-        <v>40</v>
-      </c>
-      <c r="B13" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s" s="10">
-        <v>41</v>
-      </c>
-      <c r="D13" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E13" t="s" s="10">
-        <v>26</v>
-      </c>
-      <c r="F13" t="s" s="10">
-        <v>39</v>
-      </c>
-      <c r="G13" t="s" s="10">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" t="s" s="8">
-        <v>42</v>
-      </c>
-      <c r="B14" t="s" s="9">
-        <v>9</v>
-      </c>
-      <c r="C14" t="s" s="10">
-        <v>43</v>
-      </c>
-      <c r="D14" s="11">
-        <v>5551112233</v>
-      </c>
-      <c r="E14" t="s" s="10">
-        <v>29</v>
-      </c>
-      <c r="F14" t="s" s="10">
-        <v>39</v>
-      </c>
-      <c r="G14" t="s" s="10">
-        <v>13</v>
-      </c>
+      <c r="E15" t="s" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" ht="20.05" customHeight="1">
+      <c r="A16" s="10"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+    </row>
+    <row r="17" ht="20.05" customHeight="1">
+      <c r="A17" s="10"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+    </row>
+    <row r="18" ht="20.05" customHeight="1">
+      <c r="A18" s="10"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" location="" tooltip="" display="ayse@example.test"/>
-    <hyperlink ref="C4" r:id="rId2" location="" tooltip="" display="fatma@example.test"/>
-    <hyperlink ref="C5" r:id="rId3" location="" tooltip="" display="mehmet@example.test"/>
-    <hyperlink ref="C6" r:id="rId4" location="" tooltip="" display="hikmet@example.test"/>
-    <hyperlink ref="C7" r:id="rId5" location="" tooltip="" display="ali@example.test"/>
-    <hyperlink ref="C8" r:id="rId6" location="" tooltip="" display="ahmet@example.test"/>
-    <hyperlink ref="C9" r:id="rId7" location="" tooltip="" display="ömer@example.test"/>
-    <hyperlink ref="C10" r:id="rId8" location="" tooltip="" display="nuri@example.test"/>
-    <hyperlink ref="C11" r:id="rId9" location="" tooltip="" display="hasan@example.test"/>
-    <hyperlink ref="C12" r:id="rId10" location="" tooltip="" display="cem@example.test"/>
-    <hyperlink ref="C13" r:id="rId11" location="" tooltip="" display="sultan@example.test"/>
-  </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
   <headerFooter>

</xml_diff>